<commit_message>
FIX: Uses mock-time to test templates
Uses a _different_ file to test extList styles
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/weekly_timesheet.xlsx
+++ b/xlsx/tests/templates/weekly_timesheet.xlsx
@@ -1,26 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_3290D71D983AE7626D3B866BDA9B128137D8923A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FFAAD97-09A4-47E3-8D39-5601085AEDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Timesheet" sheetId="3" r:id="rId1"/>
     <sheet name="Overview" sheetId="4" r:id="rId2"/>
+    <sheet name="METADATA" sheetId="5" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="start_date">Timesheet!$I$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -59,11 +63,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>Weekly Timesheet</t>
   </si>
   <si>
+    <t>Start date</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -82,6 +89,12 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Month overview</t>
+  </si>
+  <si>
+    <t>Week</t>
+  </si>
+  <si>
     <t>Mon</t>
   </si>
   <si>
@@ -97,25 +110,19 @@
     <t>Fri</t>
   </si>
   <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Total Monthly</t>
+  </si>
+  <si>
+    <t>By project</t>
+  </si>
+  <si>
     <t>Share</t>
   </si>
   <si>
-    <t>Week</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Start date</t>
-  </si>
-  <si>
-    <t>Total Monthly</t>
-  </si>
-  <si>
-    <t>By project</t>
-  </si>
-  <si>
-    <t>Month overview</t>
+    <t>NOW</t>
   </si>
 </sst>
 </file>
@@ -128,7 +135,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00;;\–"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -410,7 +417,7 @@
   <a:themeElements>
     <a:clrScheme name="IronCalc">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="272525"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
         <a:sysClr val="window" lastClr="FFFFFF"/>
@@ -723,17 +730,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="9" style="3" customWidth="1"/>
     <col min="2" max="2" width="9" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="33.83203125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="9.1640625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="27.75" customHeight="1">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -741,55 +748,55 @@
       <c r="C1" s="16"/>
       <c r="D1" s="32"/>
       <c r="E1" s="17" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F1" s="42">
         <f ca="1">TODAY()</f>
-        <v>46198</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="A2" s="33" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" s="34" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1">
       <c r="A3" s="35" cm="1">
-        <f t="array" aca="1" ref="A3:A32" ca="1">F1+_xlfn.SEQUENCE(DAY(EOMONTH(F1,0)))-1</f>
-        <v>46198</v>
+        <f t="array" aca="1" ref="A3:A33" ca="1">F1+_xlfn.SEQUENCE(DAY(EOMONTH(F1,0)))-1</f>
+        <v>46206</v>
       </c>
       <c r="B3" s="36" t="str" cm="1">
-        <f t="array" aca="1" ref="B3:B32" ca="1">TEXT(_xlfn.ANCHORARRAY(A3),"ddd")</f>
-        <v>ddd</v>
+        <f t="array" aca="1" ref="B3:B33" ca="1">TEXT(_xlfn.ANCHORARRAY(A3),"ddd")</f>
+        <v>Fri</v>
       </c>
       <c r="C3" s="36"/>
       <c r="D3" s="37"/>
       <c r="E3" s="38"/>
       <c r="F3" s="36"/>
     </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="18" customHeight="1">
       <c r="A4" s="35">
         <f ca="1"/>
-        <v>46199</v>
+        <v>46207</v>
       </c>
       <c r="B4" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sat</v>
       </c>
       <c r="C4" s="36"/>
       <c r="D4" s="37"/>
@@ -797,401 +804,407 @@
       <c r="F4" s="36"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="18" customHeight="1">
       <c r="A5" s="35">
         <f ca="1"/>
-        <v>46200</v>
+        <v>46208</v>
       </c>
       <c r="B5" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sun</v>
       </c>
       <c r="C5" s="36"/>
       <c r="D5" s="37"/>
       <c r="E5" s="38"/>
       <c r="F5" s="36"/>
     </row>
-    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="18" customHeight="1">
       <c r="A6" s="35">
         <f ca="1"/>
-        <v>46201</v>
+        <v>46209</v>
       </c>
       <c r="B6" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Mon</v>
       </c>
       <c r="C6" s="36"/>
       <c r="D6" s="37"/>
       <c r="E6" s="38"/>
       <c r="F6" s="36"/>
     </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="18" customHeight="1">
       <c r="A7" s="35">
         <f ca="1"/>
-        <v>46202</v>
+        <v>46210</v>
       </c>
       <c r="B7" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Tue</v>
       </c>
       <c r="C7" s="36"/>
       <c r="D7" s="37"/>
       <c r="E7" s="38"/>
       <c r="F7" s="36"/>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="18" customHeight="1">
       <c r="A8" s="35">
         <f ca="1"/>
-        <v>46203</v>
+        <v>46211</v>
       </c>
       <c r="B8" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Wed</v>
       </c>
       <c r="C8" s="39"/>
       <c r="D8" s="40"/>
       <c r="E8" s="41"/>
       <c r="F8" s="39"/>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="18" customHeight="1">
       <c r="A9" s="35">
         <f ca="1"/>
-        <v>46204</v>
+        <v>46212</v>
       </c>
       <c r="B9" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Thu</v>
       </c>
       <c r="C9" s="39"/>
       <c r="D9" s="40"/>
       <c r="E9" s="41"/>
       <c r="F9" s="39"/>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="18" customHeight="1">
       <c r="A10" s="35">
         <f ca="1"/>
-        <v>46205</v>
+        <v>46213</v>
       </c>
       <c r="B10" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Fri</v>
       </c>
       <c r="C10" s="39"/>
       <c r="D10" s="40"/>
       <c r="E10" s="41"/>
       <c r="F10" s="39"/>
     </row>
-    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="18" customHeight="1">
       <c r="A11" s="35">
         <f ca="1"/>
-        <v>46206</v>
+        <v>46214</v>
       </c>
       <c r="B11" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sat</v>
       </c>
       <c r="C11" s="39"/>
       <c r="D11" s="37"/>
       <c r="E11" s="41"/>
       <c r="F11" s="39"/>
     </row>
-    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="18" customHeight="1">
       <c r="A12" s="35">
         <f ca="1"/>
-        <v>46207</v>
+        <v>46215</v>
       </c>
       <c r="B12" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sun</v>
       </c>
       <c r="C12" s="39"/>
       <c r="D12" s="40"/>
       <c r="E12" s="41"/>
       <c r="F12" s="39"/>
     </row>
-    <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="18" customHeight="1">
       <c r="A13" s="35">
         <f ca="1"/>
-        <v>46208</v>
+        <v>46216</v>
       </c>
       <c r="B13" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Mon</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="40"/>
       <c r="E13" s="41"/>
       <c r="F13" s="39"/>
     </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="18" customHeight="1">
       <c r="A14" s="35">
         <f ca="1"/>
-        <v>46209</v>
+        <v>46217</v>
       </c>
       <c r="B14" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Tue</v>
       </c>
       <c r="C14" s="39"/>
       <c r="D14" s="40"/>
       <c r="E14" s="41"/>
       <c r="F14" s="39"/>
     </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="18" customHeight="1">
       <c r="A15" s="35">
         <f ca="1"/>
-        <v>46210</v>
+        <v>46218</v>
       </c>
       <c r="B15" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Wed</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="40"/>
       <c r="E15" s="41"/>
       <c r="F15" s="39"/>
     </row>
-    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="18" customHeight="1">
       <c r="A16" s="35">
         <f ca="1"/>
-        <v>46211</v>
+        <v>46219</v>
       </c>
       <c r="B16" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Thu</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="40"/>
       <c r="E16" s="41"/>
       <c r="F16" s="39"/>
     </row>
-    <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="18" customHeight="1">
       <c r="A17" s="35">
         <f ca="1"/>
-        <v>46212</v>
+        <v>46220</v>
       </c>
       <c r="B17" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Fri</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="40"/>
       <c r="E17" s="41"/>
       <c r="F17" s="39"/>
     </row>
-    <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="18" customHeight="1">
       <c r="A18" s="35">
         <f ca="1"/>
-        <v>46213</v>
+        <v>46221</v>
       </c>
       <c r="B18" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sat</v>
       </c>
       <c r="C18" s="39"/>
       <c r="D18" s="40"/>
       <c r="E18" s="41"/>
       <c r="F18" s="39"/>
     </row>
-    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="18" customHeight="1">
       <c r="A19" s="35">
         <f ca="1"/>
-        <v>46214</v>
+        <v>46222</v>
       </c>
       <c r="B19" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sun</v>
       </c>
       <c r="C19" s="39"/>
       <c r="D19" s="40"/>
       <c r="E19" s="41"/>
       <c r="F19" s="39"/>
     </row>
-    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="18" customHeight="1">
       <c r="A20" s="35">
         <f ca="1"/>
-        <v>46215</v>
+        <v>46223</v>
       </c>
       <c r="B20" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Mon</v>
       </c>
       <c r="C20" s="39"/>
       <c r="D20" s="40"/>
       <c r="E20" s="41"/>
       <c r="F20" s="39"/>
     </row>
-    <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="18" customHeight="1">
       <c r="A21" s="35">
         <f ca="1"/>
-        <v>46216</v>
+        <v>46224</v>
       </c>
       <c r="B21" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Tue</v>
       </c>
       <c r="C21" s="39"/>
       <c r="D21" s="40"/>
       <c r="E21" s="41"/>
       <c r="F21" s="39"/>
     </row>
-    <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="18" customHeight="1">
       <c r="A22" s="35">
         <f ca="1"/>
-        <v>46217</v>
+        <v>46225</v>
       </c>
       <c r="B22" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Wed</v>
       </c>
       <c r="C22" s="39"/>
       <c r="D22" s="40"/>
       <c r="E22" s="41"/>
       <c r="F22" s="39"/>
     </row>
-    <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="18" customHeight="1">
       <c r="A23" s="35">
         <f ca="1"/>
-        <v>46218</v>
+        <v>46226</v>
       </c>
       <c r="B23" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Thu</v>
       </c>
       <c r="C23" s="39"/>
       <c r="D23" s="40"/>
       <c r="E23" s="41"/>
       <c r="F23" s="39"/>
     </row>
-    <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="18" customHeight="1">
       <c r="A24" s="35">
         <f ca="1"/>
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B24" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Fri</v>
       </c>
       <c r="C24" s="39"/>
       <c r="D24" s="40"/>
       <c r="E24" s="41"/>
       <c r="F24" s="39"/>
     </row>
-    <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="18" customHeight="1">
       <c r="A25" s="35">
         <f ca="1"/>
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B25" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sat</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="40"/>
       <c r="E25" s="41"/>
       <c r="F25" s="39"/>
     </row>
-    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="18" customHeight="1">
       <c r="A26" s="35">
         <f ca="1"/>
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B26" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sun</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="40"/>
       <c r="E26" s="41"/>
       <c r="F26" s="39"/>
     </row>
-    <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="18" customHeight="1">
       <c r="A27" s="35">
         <f ca="1"/>
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B27" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Mon</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="40"/>
       <c r="E27" s="41"/>
       <c r="F27" s="39"/>
     </row>
-    <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="18" customHeight="1">
       <c r="A28" s="35">
         <f ca="1"/>
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B28" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Tue</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="40"/>
       <c r="E28" s="41"/>
       <c r="F28" s="39"/>
     </row>
-    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18" customHeight="1">
       <c r="A29" s="35">
         <f ca="1"/>
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B29" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Wed</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="40"/>
       <c r="E29" s="41"/>
       <c r="F29" s="39"/>
     </row>
-    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="18" customHeight="1">
       <c r="A30" s="35">
         <f ca="1"/>
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B30" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Thu</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="40"/>
       <c r="E30" s="41"/>
       <c r="F30" s="39"/>
     </row>
-    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="18" customHeight="1">
       <c r="A31" s="35">
         <f ca="1"/>
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B31" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Fri</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="40"/>
       <c r="E31" s="41"/>
       <c r="F31" s="39"/>
     </row>
-    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="18" customHeight="1">
       <c r="A32" s="35">
         <f ca="1"/>
-        <v>46227</v>
+        <v>46235</v>
       </c>
       <c r="B32" s="36" t="str">
         <f ca="1"/>
-        <v>ddd</v>
+        <v>Sat</v>
       </c>
       <c r="C32" s="39"/>
       <c r="D32" s="40"/>
       <c r="E32" s="41"/>
       <c r="F32" s="39"/>
     </row>
-    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="35"/>
-      <c r="B33" s="36"/>
+    <row r="33" spans="1:6" ht="18" customHeight="1">
+      <c r="A33" s="35">
+        <f ca="1"/>
+        <v>46236</v>
+      </c>
+      <c r="B33" s="36" t="str">
+        <f ca="1"/>
+        <v>Sun</v>
+      </c>
       <c r="C33" s="39"/>
       <c r="D33" s="40"/>
       <c r="E33" s="41"/>
@@ -1210,15 +1223,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H43"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" style="6" customWidth="1"/>
-    <col min="2" max="6" width="10.33203125" style="7" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" style="6" customWidth="1"/>
+    <col min="2" max="6" width="10.28515625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="13.7" customHeight="1">
       <c r="A1" s="15" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1226,30 +1239,30 @@
       <c r="E1" s="17"/>
       <c r="F1" s="18"/>
     </row>
-    <row r="2" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="13.7" customHeight="1">
       <c r="A2" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>10</v>
-      </c>
       <c r="F2" s="20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="13.7" customHeight="1">
       <c r="A3" s="9">
         <f ca="1">_xlfn.ISOWEEKNUM(Timesheet!F1)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B3" s="10" cm="1">
         <f t="array" aca="1" ref="B3" ca="1">SUMPRODUCT((_xlfn.ISOWEEKNUM(Timesheet!$A$3:$A$33)=$A3)*(WEEKDAY(Timesheet!$A$3:$A$33,2)=COLUMN()-COLUMN($A3))*Timesheet!$E$3:$E$33)</f>
@@ -1272,10 +1285,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="13.7" customHeight="1">
       <c r="A4" s="9">
         <f ca="1">A3+1</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" s="10" cm="1">
         <f t="array" aca="1" ref="B4" ca="1">SUMPRODUCT((_xlfn.ISOWEEKNUM(Timesheet!$A$3:$A$33)=$A4)*(WEEKDAY(Timesheet!$A$3:$A$33,2)=COLUMN()-COLUMN($A4))*Timesheet!$E$3:$E$33)</f>
@@ -1299,10 +1312,10 @@
       </c>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="13.7" customHeight="1">
       <c r="A5" s="9">
         <f ca="1">A4+1</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" s="10" cm="1">
         <f t="array" aca="1" ref="B5" ca="1">SUMPRODUCT((_xlfn.ISOWEEKNUM(Timesheet!$A$3:$A$33)=$A5)*(WEEKDAY(Timesheet!$A$3:$A$33,2)=COLUMN()-COLUMN($A5))*Timesheet!$E$3:$E$33)</f>
@@ -1325,10 +1338,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="13.7" customHeight="1">
       <c r="A6" s="9">
         <f ca="1">A5+1</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="10" cm="1">
         <f t="array" aca="1" ref="B6" ca="1">SUMPRODUCT((_xlfn.ISOWEEKNUM(Timesheet!$A$3:$A$33)=$A6)*(WEEKDAY(Timesheet!$A$3:$A$33,2)=COLUMN()-COLUMN($A6))*Timesheet!$E$3:$E$33)</f>
@@ -1351,10 +1364,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="13.7" customHeight="1">
       <c r="A7" s="9">
         <f ca="1">A6+1</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7" s="10" cm="1">
         <f t="array" aca="1" ref="B7" ca="1">SUMPRODUCT((_xlfn.ISOWEEKNUM(Timesheet!$A$3:$A$33)=$A7)*(WEEKDAY(Timesheet!$A$3:$A$33,2)=COLUMN()-COLUMN($A7))*Timesheet!$E$3:$E$33)</f>
@@ -1377,10 +1390,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ht="13.7" customHeight="1">
       <c r="A8" s="9">
         <f ca="1">A7+1</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" s="10" cm="1">
         <f t="array" aca="1" ref="B8" ca="1">SUMPRODUCT((_xlfn.ISOWEEKNUM(Timesheet!$A$3:$A$33)=$A8)*(WEEKDAY(Timesheet!$A$3:$A$33,2)=COLUMN()-COLUMN($A8))*Timesheet!$E$3:$E$33)</f>
@@ -1403,9 +1416,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="13.7" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" s="12">
         <f ca="1">SUM(B3:B8)</f>
@@ -1428,7 +1441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="13.7" customHeight="1">
       <c r="A10" s="13" t="s">
         <v>16</v>
       </c>
@@ -1441,7 +1454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="13.7" customHeight="1">
       <c r="A11" s="4"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1449,7 +1462,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="13.7" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>17</v>
       </c>
@@ -1459,21 +1472,21 @@
       <c r="E12" s="17"/>
       <c r="F12" s="18"/>
     </row>
-    <row r="13" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="13.7" customHeight="1">
       <c r="A13" s="22" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B13" s="23"/>
       <c r="C13" s="23"/>
       <c r="D13" s="23"/>
       <c r="E13" s="24" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="14.1" customHeight="1">
       <c r="A14" s="9" t="str" cm="1">
         <f t="array" ref="A14">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Timesheet!C3:C33,Timesheet!C3:C33&lt;&gt;"","No entries yet"))</f>
         <v>No entries yet</v>
@@ -1490,7 +1503,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="14.1" customHeight="1">
       <c r="A15" s="28"/>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
@@ -1498,7 +1511,7 @@
       <c r="E15" s="26"/>
       <c r="F15" s="27"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8">
       <c r="A16" s="9"/>
       <c r="B16" s="25"/>
       <c r="C16" s="25"/>
@@ -1506,7 +1519,7 @@
       <c r="E16" s="26"/>
       <c r="F16" s="27"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6">
       <c r="A17" s="9"/>
       <c r="B17" s="25"/>
       <c r="C17" s="25"/>
@@ -1514,7 +1527,7 @@
       <c r="E17" s="25"/>
       <c r="F17" s="29"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6">
       <c r="A18" s="9"/>
       <c r="B18" s="25"/>
       <c r="C18" s="25"/>
@@ -1522,7 +1535,7 @@
       <c r="E18" s="25"/>
       <c r="F18" s="29"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6">
       <c r="A19" s="9"/>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
@@ -1530,7 +1543,7 @@
       <c r="E19" s="25"/>
       <c r="F19" s="29"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6">
       <c r="A20" s="9"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
@@ -1538,7 +1551,7 @@
       <c r="E20" s="25"/>
       <c r="F20" s="29"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6">
       <c r="A21" s="9"/>
       <c r="B21" s="25"/>
       <c r="C21" s="25"/>
@@ -1546,7 +1559,7 @@
       <c r="E21" s="25"/>
       <c r="F21" s="29"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6">
       <c r="A22" s="9"/>
       <c r="B22" s="25"/>
       <c r="C22" s="25"/>
@@ -1554,7 +1567,7 @@
       <c r="E22" s="25"/>
       <c r="F22" s="29"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6">
       <c r="A23" s="9"/>
       <c r="B23" s="25"/>
       <c r="C23" s="25"/>
@@ -1562,7 +1575,7 @@
       <c r="E23" s="25"/>
       <c r="F23" s="29"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6">
       <c r="A24" s="30"/>
       <c r="B24" s="31"/>
       <c r="C24" s="31"/>
@@ -1570,7 +1583,7 @@
       <c r="E24" s="31"/>
       <c r="F24" s="29"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6">
       <c r="A25" s="30"/>
       <c r="B25" s="31"/>
       <c r="C25" s="31"/>
@@ -1578,7 +1591,7 @@
       <c r="E25" s="31"/>
       <c r="F25" s="29"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6">
       <c r="A26" s="30"/>
       <c r="B26" s="31"/>
       <c r="C26" s="31"/>
@@ -1586,7 +1599,7 @@
       <c r="E26" s="31"/>
       <c r="F26" s="29"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6">
       <c r="A27" s="30"/>
       <c r="B27" s="31"/>
       <c r="C27" s="31"/>
@@ -1594,7 +1607,7 @@
       <c r="E27" s="31"/>
       <c r="F27" s="29"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6">
       <c r="A28" s="30"/>
       <c r="B28" s="31"/>
       <c r="C28" s="31"/>
@@ -1602,7 +1615,7 @@
       <c r="E28" s="31"/>
       <c r="F28" s="29"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6">
       <c r="A29" s="30"/>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
@@ -1610,7 +1623,7 @@
       <c r="E29" s="31"/>
       <c r="F29" s="29"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6">
       <c r="A30" s="30"/>
       <c r="B30" s="31"/>
       <c r="C30" s="31"/>
@@ -1618,7 +1631,7 @@
       <c r="E30" s="31"/>
       <c r="F30" s="29"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6">
       <c r="A31" s="30"/>
       <c r="B31" s="31"/>
       <c r="C31" s="31"/>
@@ -1626,7 +1639,7 @@
       <c r="E31" s="31"/>
       <c r="F31" s="29"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6">
       <c r="A32" s="30"/>
       <c r="B32" s="31"/>
       <c r="C32" s="31"/>
@@ -1634,7 +1647,7 @@
       <c r="E32" s="31"/>
       <c r="F32" s="29"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" s="30"/>
       <c r="B33" s="31"/>
       <c r="C33" s="31"/>
@@ -1642,7 +1655,7 @@
       <c r="E33" s="31"/>
       <c r="F33" s="29"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" s="30"/>
       <c r="B34" s="31"/>
       <c r="C34" s="31"/>
@@ -1650,7 +1663,7 @@
       <c r="E34" s="31"/>
       <c r="F34" s="29"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" s="30"/>
       <c r="B35" s="31"/>
       <c r="C35" s="31"/>
@@ -1658,7 +1671,7 @@
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" s="30"/>
       <c r="B36" s="31"/>
       <c r="C36" s="31"/>
@@ -1666,7 +1679,7 @@
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" s="30"/>
       <c r="B37" s="31"/>
       <c r="C37" s="31"/>
@@ -1674,7 +1687,7 @@
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" s="30"/>
       <c r="B38" s="31"/>
       <c r="C38" s="31"/>
@@ -1682,7 +1695,7 @@
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" s="30"/>
       <c r="B39" s="31"/>
       <c r="C39" s="31"/>
@@ -1690,7 +1703,7 @@
       <c r="E39" s="31"/>
       <c r="F39" s="31"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" s="30"/>
       <c r="B40" s="31"/>
       <c r="C40" s="31"/>
@@ -1698,7 +1711,7 @@
       <c r="E40" s="31"/>
       <c r="F40" s="31"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6">
       <c r="A41" s="30"/>
       <c r="B41" s="31"/>
       <c r="C41" s="31"/>
@@ -1706,7 +1719,7 @@
       <c r="E41" s="31"/>
       <c r="F41" s="31"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" s="30"/>
       <c r="B42" s="31"/>
       <c r="C42" s="31"/>
@@ -1714,7 +1727,7 @@
       <c r="E42" s="31"/>
       <c r="F42" s="31"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" s="30"/>
       <c r="B43" s="31"/>
       <c r="C43" s="31"/>
@@ -1725,4 +1738,26 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B640EAD8-52A0-4F93-AD5A-CD57472B9353}">
+  <dimension ref="A2:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <f ca="1">NOW()</f>
+        <v>46206.472726736109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>